<commit_message>
Build program work breakdown structure
Adds four-level WBS across 12 water capital projects with lifecycle control accounts, work packages, standardized phase mappings, and updated project controls model.
</commit_message>
<xml_diff>
--- a/01_project_definition/data_dictionary.xlsx
+++ b/01_project_definition/data_dictionary.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -558,7 +558,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure category used for grouping and dashboard filtering</t>
+          <t>Infrastructure category used for grouping and dashboard filtering. Note: P12's category is 'Small Capital &amp; Emergency Response' — real, planned, scoped standing capital work with its own BAC, not the program contingency reserve. Truly unplanned scope changes draw from the reserve via change control, not from P12.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -592,24 +592,24 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Budget at Completion — total authorized baseline budget for the project (USD)</t>
+          <t>Budget at Completion — total authorized baseline budget for THIS PROJECT only (USD). Sums to the $88,500,000 project BAC total, which excludes the program contingency reserve.</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>22000000</t>
+          <t>20300000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>pct_of_program_budget</t>
+          <t>pct_of_project_bac_total</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Project BAC as a share of the $96.0M program BAC</t>
+          <t>This project's BAC as a share of the $88,500,000 project BAC total (P01-P12). Deliberately NOT a share of the $96,000,000 total program authorization, since the reserve isn't a project.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -689,7 +689,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Fields defined in the guide, populated starting Phase 4 (Earned Value Management)</t>
+          <t>Program-Level Budget Architecture (not per-project fields; live in 01_PROJECTS below the project table)</t>
         </is>
       </c>
     </row>
@@ -713,246 +713,322 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>pv</t>
+          <t>project_bac_total</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Planned Value — budgeted cost of work scheduled through the status date</t>
+          <t>Sum of all 12 project BACs. This is the 'BAC' used in every Phase 4 EVM rollup calculation.</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>7700000</t>
+          <t>88500000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>ev</t>
+          <t>program_contingency_reserve</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Earned Value — budgeted cost of work actually performed through the status date</t>
+          <t>Unallocated funds held at the program level, controlled by the Program Manager, for known-unknown risks within the program's risk profile. Not assigned to any project and not part of any project's BAC. Released only through an approved change request (07_CHANGES), at which point it transfers into the receiving project's BAC.</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>6600000</t>
+          <t>7500000</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>total_program_authorization</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Actual Cost — actual cumulative cost incurred through the status date</t>
+          <t>project_bac_total + program_contingency_reserve. The total dollar amount authorized/appropriated for the program by the governing body. This is a governance figure, not an EVM figure — do not use it as the denominator for CPI/SPI rollups.</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>7100000</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>cpi</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Cost Performance Index = EV / AC. Above 1.0 is favorable, below 1.0 is unfavorable.</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>0.93</t>
+          <t>96000000</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Schedule Performance Index = EV / PV. Above 1.0 is favorable, below 1.0 is unfavorable.</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>0.86</t>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Fields defined in the guide, populated starting Phase 4 (Earned Value Management)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>eac</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Estimate at Completion = BAC / CPI (simplified method, assumes current efficiency continues)</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>23655914</t>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Example</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>etc</t>
+          <t>pv</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Estimate to Complete = EAC − AC</t>
+          <t>Planned Value — budgeted cost of work scheduled through the status date</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>16555914</t>
+          <t>7700000</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>vac</t>
+          <t>ev</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Variance at Completion = BAC − EAC</t>
+          <t>Earned Value — budgeted cost of work actually performed through the status date</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>-1655914</t>
+          <t>6600000</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Actual Cost — actual cumulative cost incurred through the status date</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>7100000</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Fields defined in the guide, populated starting Phase 5 (Risk Register)</t>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>cpi</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Cost Performance Index = EV / AC. Above 1.0 is favorable, below 1.0 is unfavorable.</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0.93</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Example</t>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>spi</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Schedule Performance Index = EV / PV. Above 1.0 is favorable, below 1.0 is unfavorable.</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0.86</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>risk_id</t>
+          <t>eac</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Unique risk identifier</t>
+          <t>Estimate at Completion = BAC / CPI (simplified method, assumes current efficiency continues)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>R-014</t>
+          <t>23655914</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Estimate to Complete = EAC − AC</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>16555914</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>vac</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Variance at Completion = BAC − EAC</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>-1655914</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Fields defined in the guide, populated starting Phase 5 (Risk Register)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>risk_id</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Unique risk identifier</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>R-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>risk_score</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Inherent risk score = probability_score (1-5) × impact_score (1-5)</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>Fields defined in the guide, populated starting Phase 6 (Change Control)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>Definition</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>change_cost</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Approved or proposed budget impact of a change order (USD)</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>600000</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A39:D39"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>